<commit_message>
fixed waypoint names and double-checked across all data, fixed issues with Shannon diversity calculations
</commit_message>
<xml_diff>
--- a/floristics_data/abundance_data/abundance_data.xlsx
+++ b/floristics_data/abundance_data/abundance_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gwenr\Documents\Git\junction_floristics\floristics_data\abundance_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84E61647-63E7-4D13-8625-7E364F86BA98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02EC3540-4804-4058-B0E3-5C234418EFD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{9E5ABDAA-9D10-4F35-85B1-9FD21235C65A}"/>
   </bookViews>
@@ -1963,10 +1963,10 @@
       <c r="D2">
         <v>16</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="2" t="s">
         <v>12</v>
       </c>
       <c r="G2" t="s">
@@ -1976,7 +1976,7 @@
         <v>14</v>
       </c>
       <c r="I2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J2" t="s">
         <v>15</v>
@@ -1998,10 +1998,10 @@
       <c r="D3">
         <v>16</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="2" t="s">
         <v>18</v>
       </c>
       <c r="G3" t="s">
@@ -2011,7 +2011,7 @@
         <v>19</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J3" t="s">
         <v>20</v>
@@ -2033,10 +2033,10 @@
       <c r="D4">
         <v>16</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G4" t="s">
@@ -2046,7 +2046,7 @@
         <v>19</v>
       </c>
       <c r="I4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J4" t="s">
         <v>24</v>
@@ -2055,7 +2055,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -2068,26 +2068,26 @@
       <c r="D5">
         <v>16</v>
       </c>
-      <c r="E5" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" t="s">
-        <v>26</v>
+      <c r="E5" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>68</v>
       </c>
       <c r="G5" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="H5" t="s">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5" t="s">
         <v>28</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>29</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2103,10 +2103,10 @@
       <c r="D6">
         <v>16</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="2" t="s">
         <v>31</v>
       </c>
       <c r="G6" t="s">
@@ -2116,7 +2116,7 @@
         <v>19</v>
       </c>
       <c r="I6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J6" t="s">
         <v>33</v>
@@ -2138,10 +2138,10 @@
       <c r="D7">
         <v>16</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="2" t="s">
         <v>34</v>
       </c>
       <c r="G7" t="s">
@@ -2151,7 +2151,7 @@
         <v>19</v>
       </c>
       <c r="I7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7" t="s">
         <v>35</v>
@@ -2160,7 +2160,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:11" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -2173,26 +2173,26 @@
       <c r="D8">
         <v>16</v>
       </c>
-      <c r="E8" t="s">
-        <v>37</v>
-      </c>
-      <c r="F8" t="s">
-        <v>38</v>
+      <c r="E8" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>32</v>
       </c>
       <c r="G8" t="s">
         <v>32</v>
       </c>
       <c r="H8" t="s">
-        <v>19</v>
+        <v>71</v>
       </c>
       <c r="I8">
         <v>1</v>
       </c>
       <c r="J8" t="s">
-        <v>39</v>
+        <v>72</v>
       </c>
       <c r="K8" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2208,26 +2208,26 @@
       <c r="D9">
         <v>16</v>
       </c>
-      <c r="E9" t="s">
-        <v>41</v>
-      </c>
-      <c r="F9" t="s">
-        <v>42</v>
+      <c r="E9" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>74</v>
       </c>
       <c r="G9" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="H9" t="s">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="I9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J9" t="s">
-        <v>43</v>
+        <v>75</v>
       </c>
       <c r="K9" t="s">
-        <v>28</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2243,11 +2243,11 @@
       <c r="D10">
         <v>16</v>
       </c>
-      <c r="E10" t="s">
-        <v>44</v>
-      </c>
-      <c r="F10" t="s">
-        <v>44</v>
+      <c r="E10" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>78</v>
       </c>
       <c r="G10" t="s">
         <v>32</v>
@@ -2256,16 +2256,16 @@
         <v>19</v>
       </c>
       <c r="I10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J10" t="s">
-        <v>45</v>
+        <v>79</v>
       </c>
       <c r="K10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -2279,13 +2279,13 @@
         <v>16</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="F11" t="s">
-        <v>48</v>
+        <v>80</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>81</v>
       </c>
       <c r="G11" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="H11" t="s">
         <v>19</v>
@@ -2294,10 +2294,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="K11" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2313,23 +2313,23 @@
       <c r="D12">
         <v>16</v>
       </c>
-      <c r="E12" t="s">
-        <v>50</v>
-      </c>
-      <c r="F12" t="s">
-        <v>51</v>
+      <c r="E12" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="G12" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="H12" t="s">
         <v>19</v>
       </c>
       <c r="I12">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="J12" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="K12" t="s">
         <v>28</v>
@@ -2348,11 +2348,11 @@
       <c r="D13">
         <v>16</v>
       </c>
-      <c r="E13" t="s">
-        <v>53</v>
-      </c>
-      <c r="F13" t="s">
-        <v>53</v>
+      <c r="E13" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="G13" t="s">
         <v>32</v>
@@ -2361,13 +2361,13 @@
         <v>19</v>
       </c>
       <c r="I13">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J13" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="K13" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2383,11 +2383,11 @@
       <c r="D14">
         <v>16</v>
       </c>
-      <c r="E14" t="s">
-        <v>55</v>
+      <c r="E14" s="2" t="s">
+        <v>83</v>
       </c>
       <c r="F14" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="G14" t="s">
         <v>32</v>
@@ -2396,13 +2396,13 @@
         <v>19</v>
       </c>
       <c r="I14">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J14" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="K14" t="s">
-        <v>58</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2418,26 +2418,26 @@
       <c r="D15">
         <v>16</v>
       </c>
-      <c r="E15" t="s">
-        <v>59</v>
-      </c>
-      <c r="F15" t="s">
-        <v>60</v>
+      <c r="E15" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>85</v>
       </c>
       <c r="G15" t="s">
         <v>32</v>
       </c>
       <c r="H15" t="s">
-        <v>61</v>
+        <v>14</v>
       </c>
       <c r="I15">
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="K15" t="s">
-        <v>28</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2453,26 +2453,26 @@
       <c r="D16">
         <v>16</v>
       </c>
-      <c r="E16" t="s">
-        <v>63</v>
-      </c>
-      <c r="F16" t="s">
-        <v>64</v>
+      <c r="E16" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>53</v>
       </c>
       <c r="G16" t="s">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="H16" t="s">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="I16">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>63</v>
+        <v>28</v>
       </c>
       <c r="K16" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2488,26 +2488,26 @@
       <c r="D17">
         <v>16</v>
       </c>
-      <c r="E17" t="s">
-        <v>63</v>
+      <c r="E17" s="2" t="s">
+        <v>87</v>
       </c>
       <c r="F17" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="G17" t="s">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="H17" t="s">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="I17">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="K17" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2523,26 +2523,26 @@
       <c r="D18">
         <v>16</v>
       </c>
-      <c r="E18" t="s">
-        <v>63</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>66</v>
+      <c r="E18" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F18" t="s">
+        <v>60</v>
       </c>
       <c r="G18" t="s">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="H18" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I18">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K18" t="s">
-        <v>63</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2556,28 +2556,28 @@
         <v>2</v>
       </c>
       <c r="D19">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>12</v>
+        <v>63</v>
+      </c>
+      <c r="F19" t="s">
+        <v>64</v>
       </c>
       <c r="G19" t="s">
-        <v>13</v>
+        <v>63</v>
       </c>
       <c r="H19" t="s">
+        <v>63</v>
+      </c>
+      <c r="I19">
         <v>14</v>
       </c>
-      <c r="I19">
-        <v>7</v>
-      </c>
       <c r="J19" t="s">
-        <v>15</v>
+        <v>63</v>
       </c>
       <c r="K19" t="s">
-        <v>16</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2591,28 +2591,28 @@
         <v>2</v>
       </c>
       <c r="D20">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>18</v>
+        <v>63</v>
+      </c>
+      <c r="F20" t="s">
+        <v>65</v>
       </c>
       <c r="G20" t="s">
-        <v>13</v>
+        <v>63</v>
       </c>
       <c r="H20" t="s">
-        <v>19</v>
+        <v>63</v>
       </c>
       <c r="I20">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="J20" t="s">
-        <v>20</v>
+        <v>63</v>
       </c>
       <c r="K20" t="s">
-        <v>21</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2626,28 +2626,28 @@
         <v>2</v>
       </c>
       <c r="D21">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>23</v>
+        <v>66</v>
       </c>
       <c r="G21" t="s">
-        <v>13</v>
+        <v>63</v>
       </c>
       <c r="H21" t="s">
-        <v>19</v>
+        <v>63</v>
       </c>
       <c r="I21">
-        <v>2</v>
+        <v>58</v>
       </c>
       <c r="J21" t="s">
-        <v>24</v>
+        <v>63</v>
       </c>
       <c r="K21" t="s">
-        <v>25</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2663,26 +2663,26 @@
       <c r="D22">
         <v>33</v>
       </c>
-      <c r="E22" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>68</v>
+      <c r="E22" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" t="s">
+        <v>12</v>
       </c>
       <c r="G22" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="H22" t="s">
-        <v>61</v>
+        <v>14</v>
       </c>
       <c r="I22">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J22" t="s">
-        <v>28</v>
-      </c>
-      <c r="K22" s="2" t="s">
-        <v>69</v>
+        <v>15</v>
+      </c>
+      <c r="K22" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2698,14 +2698,14 @@
       <c r="D23">
         <v>33</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>31</v>
+      <c r="E23" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" t="s">
+        <v>18</v>
       </c>
       <c r="G23" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="H23" t="s">
         <v>19</v>
@@ -2714,10 +2714,10 @@
         <v>3</v>
       </c>
       <c r="J23" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="K23" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2733,11 +2733,11 @@
       <c r="D24">
         <v>33</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>34</v>
+      <c r="E24" t="s">
+        <v>22</v>
+      </c>
+      <c r="F24" t="s">
+        <v>23</v>
       </c>
       <c r="G24" t="s">
         <v>13</v>
@@ -2746,16 +2746,16 @@
         <v>19</v>
       </c>
       <c r="I24">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J24" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="K24" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" t="s">
         <v>10</v>
       </c>
@@ -2768,26 +2768,26 @@
       <c r="D25">
         <v>33</v>
       </c>
-      <c r="E25" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>32</v>
+      <c r="E25" t="s">
+        <v>26</v>
+      </c>
+      <c r="F25" t="s">
+        <v>26</v>
       </c>
       <c r="G25" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="H25" t="s">
-        <v>71</v>
+        <v>19</v>
       </c>
       <c r="I25">
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>72</v>
-      </c>
-      <c r="K25" t="s">
-        <v>28</v>
+        <v>28</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2803,26 +2803,26 @@
       <c r="D26">
         <v>33</v>
       </c>
-      <c r="E26" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>74</v>
+      <c r="E26" t="s">
+        <v>30</v>
+      </c>
+      <c r="F26" t="s">
+        <v>31</v>
       </c>
       <c r="G26" t="s">
         <v>32</v>
       </c>
       <c r="H26" t="s">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="I26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J26" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="K26" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2838,14 +2838,14 @@
       <c r="D27">
         <v>33</v>
       </c>
-      <c r="E27" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>78</v>
+      <c r="E27" t="s">
+        <v>34</v>
+      </c>
+      <c r="F27" t="s">
+        <v>34</v>
       </c>
       <c r="G27" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="H27" t="s">
         <v>19</v>
@@ -2854,10 +2854,10 @@
         <v>2</v>
       </c>
       <c r="J27" t="s">
-        <v>79</v>
+        <v>35</v>
       </c>
       <c r="K27" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2873,11 +2873,11 @@
       <c r="D28">
         <v>33</v>
       </c>
-      <c r="E28" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>81</v>
+      <c r="E28" t="s">
+        <v>37</v>
+      </c>
+      <c r="F28" t="s">
+        <v>38</v>
       </c>
       <c r="G28" t="s">
         <v>32</v>
@@ -2889,10 +2889,10 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="K28" t="s">
-        <v>82</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -2908,10 +2908,10 @@
       <c r="D29">
         <v>33</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="E29" t="s">
         <v>41</v>
       </c>
-      <c r="F29" s="2" t="s">
+      <c r="F29" t="s">
         <v>42</v>
       </c>
       <c r="G29" t="s">
@@ -2921,7 +2921,7 @@
         <v>19</v>
       </c>
       <c r="I29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J29" t="s">
         <v>43</v>
@@ -2943,10 +2943,10 @@
       <c r="D30">
         <v>33</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="E30" t="s">
         <v>44</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="F30" t="s">
         <v>44</v>
       </c>
       <c r="G30" t="s">
@@ -2956,7 +2956,7 @@
         <v>19</v>
       </c>
       <c r="I30">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J30" t="s">
         <v>45</v>
@@ -2965,7 +2965,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:11" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
         <v>10</v>
       </c>
@@ -2979,22 +2979,22 @@
         <v>33</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>83</v>
+        <v>47</v>
       </c>
       <c r="F31" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G31" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="H31" t="s">
         <v>19</v>
       </c>
       <c r="I31">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="K31" t="s">
         <v>28</v>
@@ -3013,26 +3013,26 @@
       <c r="D32">
         <v>33</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>85</v>
+      <c r="E32" t="s">
+        <v>50</v>
+      </c>
+      <c r="F32" t="s">
+        <v>51</v>
       </c>
       <c r="G32" t="s">
         <v>32</v>
       </c>
       <c r="H32" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="I32">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="J32" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="K32" t="s">
-        <v>86</v>
+        <v>28</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -3048,10 +3048,10 @@
       <c r="D33">
         <v>33</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="E33" t="s">
         <v>53</v>
       </c>
-      <c r="F33" s="2" t="s">
+      <c r="F33" t="s">
         <v>53</v>
       </c>
       <c r="G33" t="s">
@@ -3083,8 +3083,8 @@
       <c r="D34">
         <v>33</v>
       </c>
-      <c r="E34" s="2" t="s">
-        <v>87</v>
+      <c r="E34" t="s">
+        <v>55</v>
       </c>
       <c r="F34" t="s">
         <v>56</v>
@@ -3118,7 +3118,7 @@
       <c r="D35">
         <v>33</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="E35" t="s">
         <v>59</v>
       </c>
       <c r="F35" t="s">
@@ -3153,7 +3153,7 @@
       <c r="D36">
         <v>33</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="E36" t="s">
         <v>63</v>
       </c>
       <c r="F36" t="s">
@@ -3166,7 +3166,7 @@
         <v>63</v>
       </c>
       <c r="I36">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="J36" t="s">
         <v>63</v>
@@ -3188,7 +3188,7 @@
       <c r="D37">
         <v>33</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="E37" t="s">
         <v>63</v>
       </c>
       <c r="F37" t="s">
@@ -3201,7 +3201,7 @@
         <v>63</v>
       </c>
       <c r="I37">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J37" t="s">
         <v>63</v>
@@ -3223,7 +3223,7 @@
       <c r="D38">
         <v>33</v>
       </c>
-      <c r="E38" s="2" t="s">
+      <c r="E38" t="s">
         <v>63</v>
       </c>
       <c r="F38" s="2" t="s">
@@ -3236,7 +3236,7 @@
         <v>63</v>
       </c>
       <c r="I38">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="J38" t="s">
         <v>63</v>
@@ -4426,7 +4426,7 @@
         <v>71</v>
       </c>
       <c r="I72">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J72" t="s">
         <v>28</v>
@@ -4531,7 +4531,7 @@
         <v>61</v>
       </c>
       <c r="I75">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J75" t="s">
         <v>171</v>
@@ -4566,7 +4566,7 @@
         <v>19</v>
       </c>
       <c r="I76">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J76" t="s">
         <v>28</v>
@@ -12766,6 +12766,9 @@
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K312">
+    <sortCondition ref="A1:A312"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
fixed habitat of transects 2 and 4, added aspect info
</commit_message>
<xml_diff>
--- a/floristics_data/abundance_data/abundance_data.xlsx
+++ b/floristics_data/abundance_data/abundance_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gwenr\Documents\Git\junction_floristics\floristics_data\abundance_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02EC3540-4804-4058-B0E3-5C234418EFD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B22C1EF1-6256-494F-AD89-BB2F00AE8DE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{9E5ABDAA-9D10-4F35-85B1-9FD21235C65A}"/>
   </bookViews>
@@ -1955,7 +1955,7 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -1990,7 +1990,7 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -2060,7 +2060,7 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C5">
         <v>2</v>
@@ -2095,7 +2095,7 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -2130,7 +2130,7 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C7">
         <v>2</v>
@@ -2165,7 +2165,7 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C8">
         <v>2</v>
@@ -2200,7 +2200,7 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C9">
         <v>2</v>
@@ -2235,7 +2235,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C10">
         <v>2</v>
@@ -2270,7 +2270,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C11">
         <v>2</v>
@@ -2305,7 +2305,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C12">
         <v>2</v>
@@ -2340,7 +2340,7 @@
         <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C13">
         <v>2</v>
@@ -2375,7 +2375,7 @@
         <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C14">
         <v>2</v>
@@ -2410,7 +2410,7 @@
         <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C15">
         <v>2</v>
@@ -2445,7 +2445,7 @@
         <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C16">
         <v>2</v>
@@ -2480,7 +2480,7 @@
         <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C17">
         <v>2</v>
@@ -2515,7 +2515,7 @@
         <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C18">
         <v>2</v>
@@ -2550,7 +2550,7 @@
         <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C19">
         <v>2</v>
@@ -2585,7 +2585,7 @@
         <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C20">
         <v>2</v>
@@ -2620,7 +2620,7 @@
         <v>10</v>
       </c>
       <c r="B21" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C21">
         <v>2</v>
@@ -2655,7 +2655,7 @@
         <v>10</v>
       </c>
       <c r="B22" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C22">
         <v>2</v>
@@ -2690,7 +2690,7 @@
         <v>10</v>
       </c>
       <c r="B23" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C23">
         <v>2</v>
@@ -2725,7 +2725,7 @@
         <v>10</v>
       </c>
       <c r="B24" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C24">
         <v>2</v>
@@ -2760,7 +2760,7 @@
         <v>10</v>
       </c>
       <c r="B25" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C25">
         <v>2</v>
@@ -2795,7 +2795,7 @@
         <v>10</v>
       </c>
       <c r="B26" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C26">
         <v>2</v>
@@ -2830,7 +2830,7 @@
         <v>10</v>
       </c>
       <c r="B27" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C27">
         <v>2</v>
@@ -2865,7 +2865,7 @@
         <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C28">
         <v>2</v>
@@ -2900,7 +2900,7 @@
         <v>10</v>
       </c>
       <c r="B29" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C29">
         <v>2</v>
@@ -2935,7 +2935,7 @@
         <v>10</v>
       </c>
       <c r="B30" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C30">
         <v>2</v>
@@ -2970,7 +2970,7 @@
         <v>10</v>
       </c>
       <c r="B31" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C31">
         <v>2</v>
@@ -3005,7 +3005,7 @@
         <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C32">
         <v>2</v>
@@ -3040,7 +3040,7 @@
         <v>10</v>
       </c>
       <c r="B33" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C33">
         <v>2</v>
@@ -3075,7 +3075,7 @@
         <v>10</v>
       </c>
       <c r="B34" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C34">
         <v>2</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="B35" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C35">
         <v>2</v>
@@ -3145,7 +3145,7 @@
         <v>10</v>
       </c>
       <c r="B36" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C36">
         <v>2</v>
@@ -3180,7 +3180,7 @@
         <v>10</v>
       </c>
       <c r="B37" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C37">
         <v>2</v>
@@ -3215,7 +3215,7 @@
         <v>10</v>
       </c>
       <c r="B38" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="C38">
         <v>2</v>
@@ -3250,7 +3250,7 @@
         <v>10</v>
       </c>
       <c r="B39" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="C39">
         <v>4</v>
@@ -3285,7 +3285,7 @@
         <v>10</v>
       </c>
       <c r="B40" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="C40">
         <v>4</v>
@@ -3320,7 +3320,7 @@
         <v>10</v>
       </c>
       <c r="B41" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="C41">
         <v>4</v>
@@ -3355,7 +3355,7 @@
         <v>10</v>
       </c>
       <c r="B42" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="C42">
         <v>4</v>
@@ -3390,7 +3390,7 @@
         <v>10</v>
       </c>
       <c r="B43" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="C43">
         <v>4</v>
@@ -3425,7 +3425,7 @@
         <v>10</v>
       </c>
       <c r="B44" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="C44">
         <v>4</v>
@@ -3460,7 +3460,7 @@
         <v>10</v>
       </c>
       <c r="B45" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="C45">
         <v>4</v>
@@ -3495,7 +3495,7 @@
         <v>10</v>
       </c>
       <c r="B46" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="C46">
         <v>4</v>
@@ -3530,7 +3530,7 @@
         <v>10</v>
       </c>
       <c r="B47" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="C47">
         <v>4</v>
@@ -3565,7 +3565,7 @@
         <v>10</v>
       </c>
       <c r="B48" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="C48">
         <v>4</v>
@@ -3600,7 +3600,7 @@
         <v>10</v>
       </c>
       <c r="B49" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="C49">
         <v>4</v>
@@ -3635,7 +3635,7 @@
         <v>10</v>
       </c>
       <c r="B50" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="C50">
         <v>4</v>
@@ -3670,7 +3670,7 @@
         <v>10</v>
       </c>
       <c r="B51" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="C51">
         <v>4</v>
@@ -3705,7 +3705,7 @@
         <v>10</v>
       </c>
       <c r="B52" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="C52">
         <v>4</v>

</xml_diff>